<commit_message>
Updated PRD and Excel of Variables for dashboard updates
all changes to both documents have been highlighted in Yellow
</commit_message>
<xml_diff>
--- a/Data/data documentation/Data documentation for council variables.xlsx
+++ b/Data/data documentation/Data documentation for council variables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\Github\philadelphia-council-districts-and-health\Data\data documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{925B5796-3466-4522-AE1C-06CF5B143E71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01B3F741-F830-43A2-8E49-C5302E8723C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{7E76C4D9-7630-4340-BEBA-4E6127603C3B}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="159">
   <si>
     <t>Map</t>
   </si>
@@ -488,9 +488,6 @@
     <t>Census Tract aggregated up to the council district using Block population as weights</t>
   </si>
   <si>
-    <t>Count of Licenses</t>
-  </si>
-  <si>
     <t>Counts already at the council district level</t>
   </si>
   <si>
@@ -507,12 +504,6 @@
   </si>
   <si>
     <t xml:space="preserve">Code violations were set at the council district level. However land parcels had to be spatially joined to council districts. </t>
-  </si>
-  <si>
-    <t>Percentage of homes that lack a complete kitchen</t>
-  </si>
-  <si>
-    <t>Percentage of homes that lack complete plumbing</t>
   </si>
   <si>
     <t>Census Block Group aggregated up to the council district using total number of households as weights</t>
@@ -607,6 +598,18 @@
   </si>
   <si>
     <t>Percentage of residents who are two or more races</t>
+  </si>
+  <si>
+    <t>Percentage of homes that lack a complete kitchen. A housing unit is considered to be lacking complete kitchen facilities when it is missing one or more of the following: a sink with a faucet, a stove or range, and a refrigerator.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Percentage of homes that lack complete plumbing. A housing unit is considered to be lacking complete plumbing facilities when it is missing one or more of the following: hot and cold running water and a bathtub or shower. </t>
+  </si>
+  <si>
+    <t>Count of Licenses. Non-rental Business Licenses are for business that do not involve leasing property such as restaurants, retail stores, street vendors, contractors, and other professional services.</t>
+  </si>
+  <si>
+    <t>Count of Licenses. Rental business licenses are required for business that involves leasing property (both residential and commercial) including landlord properties, assisted living facilities, hotels, and dormitories.</t>
   </si>
 </sst>
 </file>
@@ -769,7 +772,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -947,6 +950,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1110,7 +1119,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1131,6 +1140,9 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1949,12 +1961,12 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="156" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>123</v>
+      <c r="B4" s="10" t="s">
+        <v>157</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>65</v>
@@ -1966,15 +1978,15 @@
         <v>43</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>123</v>
+      <c r="B5" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>65</v>
@@ -1986,7 +1998,7 @@
         <v>43</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
@@ -1994,7 +2006,7 @@
         <v>30</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>65</v>
@@ -2006,7 +2018,7 @@
         <v>32</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="280.8" x14ac:dyDescent="0.3">
@@ -2106,10 +2118,10 @@
         <v>79</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>128</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>8</v>
@@ -2118,18 +2130,18 @@
         <v>51</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>130</v>
+      <c r="B12" s="10" t="s">
+        <v>155</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>67</v>
@@ -2141,18 +2153,18 @@
         <v>122</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>131</v>
+      <c r="B13" s="10" t="s">
+        <v>156</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>67</v>
@@ -2164,7 +2176,7 @@
         <v>122</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
@@ -2184,10 +2196,10 @@
         <v>66</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
@@ -2195,10 +2207,10 @@
         <v>83</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>67</v>
@@ -2207,10 +2219,10 @@
         <v>66</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
@@ -2218,10 +2230,10 @@
         <v>84</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>67</v>
@@ -2230,10 +2242,10 @@
         <v>66</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="78" x14ac:dyDescent="0.3">
@@ -2264,7 +2276,7 @@
         <v>86</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>108</v>
@@ -2287,7 +2299,7 @@
         <v>87</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>108</v>
@@ -2310,7 +2322,7 @@
         <v>88</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>108</v>
@@ -2333,7 +2345,7 @@
         <v>89</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>108</v>
@@ -2356,7 +2368,7 @@
         <v>90</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>108</v>
@@ -2379,7 +2391,7 @@
         <v>91</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>108</v>
@@ -2425,7 +2437,7 @@
         <v>93</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>65</v>
@@ -2437,7 +2449,7 @@
         <v>47</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
@@ -2445,7 +2457,7 @@
         <v>94</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>65</v>
@@ -2457,7 +2469,7 @@
         <v>47</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
@@ -2465,10 +2477,10 @@
         <v>95</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="D27" s="7" t="s">
         <v>67</v>
@@ -2477,10 +2489,10 @@
         <v>66</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="109.2" x14ac:dyDescent="0.3">
@@ -2488,10 +2500,10 @@
         <v>96</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>36</v>
@@ -2500,10 +2512,10 @@
         <v>2019</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="109.2" x14ac:dyDescent="0.3">
@@ -2523,10 +2535,10 @@
         <v>2018</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="78" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
updated the PRD and excel doc with edits that need to be made by @ran-codes
</commit_message>
<xml_diff>
--- a/Data/data documentation/Data documentation for council variables.xlsx
+++ b/Data/data documentation/Data documentation for council variables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\Github\philadelphia-council-districts-and-health\Data\data documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://drexel0-my.sharepoint.com/personal/tr842_drexel_edu/Documents/Github_repositories/philadelphia-council-districts-and-health/Data/data documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01B3F741-F830-43A2-8E49-C5302E8723C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{01B3F741-F830-43A2-8E49-C5302E8723C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB51266C-89A8-4746-98C8-07184BF99B7F}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{7E76C4D9-7630-4340-BEBA-4E6127603C3B}"/>
+    <workbookView xWindow="6600" yWindow="2760" windowWidth="23260" windowHeight="12460" activeTab="1" xr2:uid="{7E76C4D9-7630-4340-BEBA-4E6127603C3B}"/>
   </bookViews>
   <sheets>
     <sheet name="Data documentation for council " sheetId="1" r:id="rId1"/>
@@ -594,9 +594,6 @@
     <t>Percentage of residents who are Pacific Islander/Native Hawaiian</t>
   </si>
   <si>
-    <t>Percentage of residents who are other race</t>
-  </si>
-  <si>
     <t>Percentage of residents who are two or more races</t>
   </si>
   <si>
@@ -610,6 +607,9 @@
   </si>
   <si>
     <t>Count of Licenses. Rental business licenses are required for business that involves leasing property (both residential and commercial) including landlord properties, assisted living facilities, hotels, and dormitories.</t>
+  </si>
+  <si>
+    <t>Percentage of residents who identified with a race other than the listed racial categories</t>
   </si>
 </sst>
 </file>
@@ -1199,6 +1199,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1519,18 +1523,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01CB8890-B7A9-3A40-979C-A48DC9A37105}">
   <dimension ref="A1:H27"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.19921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.296875" customWidth="1"/>
-    <col min="6" max="6" width="27.19921875" customWidth="1"/>
-    <col min="7" max="7" width="15.19921875" customWidth="1"/>
+    <col min="2" max="2" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.33203125" customWidth="1"/>
+    <col min="6" max="6" width="27.1640625" customWidth="1"/>
+    <col min="7" max="7" width="15.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1553,7 +1557,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1576,7 +1580,7 @@
         <v>45716</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="265.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="289" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1599,7 +1603,7 @@
         <v>45725</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="358.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="388" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -1622,7 +1626,7 @@
         <v>45726</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="187.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="204" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -1645,7 +1649,7 @@
         <v>45718</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -1668,7 +1672,7 @@
         <v>45719</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>27</v>
       </c>
@@ -1691,7 +1695,7 @@
         <v>45719</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -1714,7 +1718,7 @@
         <v>45719</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>35</v>
       </c>
@@ -1734,7 +1738,7 @@
         <v>45719</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>38</v>
       </c>
@@ -1757,7 +1761,7 @@
         <v>45725</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -1780,7 +1784,7 @@
         <v>45725</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>46</v>
       </c>
@@ -1803,7 +1807,7 @@
         <v>45726</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>50</v>
       </c>
@@ -1826,7 +1830,7 @@
         <v>45725</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="296.39999999999998" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="323" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>54</v>
       </c>
@@ -1849,7 +1853,7 @@
         <v>45726</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="187.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="221" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>57</v>
       </c>
@@ -1872,7 +1876,7 @@
         <v>45726</v>
       </c>
     </row>
-    <row r="26" spans="1:8" s="5" customFormat="1" ht="19.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" s="5" customFormat="1" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -1882,7 +1886,7 @@
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -1900,17 +1904,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B07AACCA-88DB-7C45-AECA-8998520502A5}">
   <dimension ref="A1:G30"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.19921875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="20.296875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="22.296875" style="2" customWidth="1"/>
-    <col min="4" max="5" width="11.19921875" style="2"/>
-    <col min="6" max="6" width="19.69921875" customWidth="1"/>
+    <col min="1" max="1" width="20.1640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.33203125" style="2" customWidth="1"/>
+    <col min="4" max="5" width="11.1640625" style="2"/>
+    <col min="6" max="6" width="19.6640625" customWidth="1"/>
     <col min="7" max="7" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>60</v>
       </c>
@@ -1933,7 +1937,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
         <v>20</v>
       </c>
@@ -1956,17 +1960,17 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="156" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="170" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>65</v>
@@ -1981,12 +1985,12 @@
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="171.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="187" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>74</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>65</v>
@@ -2001,7 +2005,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>30</v>
       </c>
@@ -2021,7 +2025,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="280.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="306" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>78</v>
       </c>
@@ -2044,7 +2048,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>77</v>
       </c>
@@ -2067,7 +2071,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="119" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>75</v>
       </c>
@@ -2090,7 +2094,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="119" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>76</v>
       </c>
@@ -2113,7 +2117,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>79</v>
       </c>
@@ -2133,12 +2137,12 @@
         <v>128</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="171.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="187" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>80</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>132</v>
@@ -2156,12 +2160,12 @@
         <v>131</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="171.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="187" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>132</v>
@@ -2179,7 +2183,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>82</v>
       </c>
@@ -2202,7 +2206,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>83</v>
       </c>
@@ -2225,7 +2229,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>84</v>
       </c>
@@ -2248,7 +2252,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>85</v>
       </c>
@@ -2271,7 +2275,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>86</v>
       </c>
@@ -2294,7 +2298,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>87</v>
       </c>
@@ -2317,7 +2321,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>88</v>
       </c>
@@ -2340,7 +2344,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>89</v>
       </c>
@@ -2363,12 +2367,12 @@
         <v>113</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>153</v>
+      <c r="B22" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>108</v>
@@ -2386,12 +2390,12 @@
         <v>114</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>91</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>108</v>
@@ -2409,7 +2413,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>92</v>
       </c>
@@ -2432,7 +2436,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>93</v>
       </c>
@@ -2452,7 +2456,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>94</v>
       </c>
@@ -2472,7 +2476,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>95</v>
       </c>
@@ -2495,7 +2499,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" ht="119" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>96</v>
       </c>
@@ -2518,7 +2522,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" ht="119" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>97</v>
       </c>
@@ -2541,7 +2545,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>57</v>
       </c>

</xml_diff>

<commit_message>
Updated the excel document
</commit_message>
<xml_diff>
--- a/Data/data documentation/Data documentation for council variables.xlsx
+++ b/Data/data documentation/Data documentation for council variables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://drexel0-my.sharepoint.com/personal/tr842_drexel_edu/Documents/Github_repositories/philadelphia-council-districts-and-health/Data/data documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{01B3F741-F830-43A2-8E49-C5302E8723C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB51266C-89A8-4746-98C8-07184BF99B7F}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{01B3F741-F830-43A2-8E49-C5302E8723C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF151C33-62E8-0F4B-868C-E4FB1A4C9C84}"/>
   <bookViews>
     <workbookView xWindow="6600" yWindow="2760" windowWidth="23260" windowHeight="12460" activeTab="1" xr2:uid="{7E76C4D9-7630-4340-BEBA-4E6127603C3B}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="164">
   <si>
     <t>Map</t>
   </si>
@@ -610,6 +610,21 @@
   </si>
   <si>
     <t>Percentage of residents who identified with a race other than the listed racial categories</t>
+  </si>
+  <si>
+    <t>Open Data Philly (Department of Licenses and Inspections)</t>
+  </si>
+  <si>
+    <t>Open Data Philly (Philadelphia Police Department)</t>
+  </si>
+  <si>
+    <t>Urban Health Collaborative Data Portal</t>
+  </si>
+  <si>
+    <t>Open Data Philly (Department of Public Health)</t>
+  </si>
+  <si>
+    <t>Total number of people in the district</t>
   </si>
 </sst>
 </file>
@@ -1119,7 +1134,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1141,6 +1156,9 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1960,9 +1978,24 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>72</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="170" x14ac:dyDescent="0.2">
@@ -1975,8 +2008,8 @@
       <c r="C4" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>8</v>
+      <c r="D4" s="10" t="s">
+        <v>159</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>43</v>
@@ -1995,8 +2028,8 @@
       <c r="C5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>8</v>
+      <c r="D5" s="10" t="s">
+        <v>159</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>43</v>
@@ -2005,7 +2038,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>30</v>
       </c>
@@ -2015,8 +2048,8 @@
       <c r="C6" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>8</v>
+      <c r="D6" s="10" t="s">
+        <v>160</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>32</v>
@@ -2127,8 +2160,8 @@
       <c r="C11" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>8</v>
+      <c r="D11" s="10" t="s">
+        <v>159</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>51</v>
@@ -2436,7 +2469,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>93</v>
       </c>
@@ -2446,8 +2479,8 @@
       <c r="C25" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>8</v>
+      <c r="D25" s="10" t="s">
+        <v>160</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>47</v>
@@ -2456,7 +2489,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>94</v>
       </c>
@@ -2466,8 +2499,8 @@
       <c r="C26" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>8</v>
+      <c r="D26" s="10" t="s">
+        <v>160</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>47</v>
@@ -2476,7 +2509,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>95</v>
       </c>
@@ -2509,8 +2542,8 @@
       <c r="C28" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>36</v>
+      <c r="D28" s="10" t="s">
+        <v>161</v>
       </c>
       <c r="E28" s="2">
         <v>2019</v>
@@ -2532,8 +2565,8 @@
       <c r="C29" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>8</v>
+      <c r="D29" s="10" t="s">
+        <v>162</v>
       </c>
       <c r="E29" s="2">
         <v>2018</v>

</xml_diff>

<commit_message>
fixing spelling of vulnerability
</commit_message>
<xml_diff>
--- a/Data/data documentation/Data documentation for council variables.xlsx
+++ b/Data/data documentation/Data documentation for council variables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://drexel0-my.sharepoint.com/personal/tr842_drexel_edu/Documents/Github_repositories/philadelphia-council-districts-and-health/Data/data documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{01B3F741-F830-43A2-8E49-C5302E8723C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF151C33-62E8-0F4B-868C-E4FB1A4C9C84}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{01B3F741-F830-43A2-8E49-C5302E8723C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D2CF2A3-1FAC-AB46-9E38-E583BFA9D6A2}"/>
   <bookViews>
     <workbookView xWindow="6600" yWindow="2760" windowWidth="23260" windowHeight="12460" activeTab="1" xr2:uid="{7E76C4D9-7630-4340-BEBA-4E6127603C3B}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="163">
   <si>
     <t>Map</t>
   </si>
@@ -363,9 +363,6 @@
     <t>Tree Canopy Coverage</t>
   </si>
   <si>
-    <t>Heat Vulnerabillity Index</t>
-  </si>
-  <si>
     <t xml:space="preserve">Variables Used: 
 #"B15003_001" = total pop over 25
 #"B15003_002" = No schooling
@@ -429,11 +426,6 @@
   </si>
   <si>
     <t>Variables Used:
-#B02001_001 Total pop
-#B03002_003 White Not hispanic or Latino</t>
-  </si>
-  <si>
-    <t>Variables Used:
 #B02001_001 Total pop,
 #B02001_003 Black</t>
   </si>
@@ -466,9 +458,6 @@
     <t>Variables Used:
 #B03001_001 Total pop,
 #B03002_012 Hispanic/Latino</t>
-  </si>
-  <si>
-    <t>Percentage of residents who are White, Non-hispanic</t>
   </si>
   <si>
     <t>Percentage of residents who are Hispanic</t>
@@ -625,6 +614,14 @@
   </si>
   <si>
     <t>Total number of people in the district</t>
+  </si>
+  <si>
+    <t>Percentage of residents who are White, Non-Hispanic</t>
+  </si>
+  <si>
+    <t>Variables Used:
+#B02001_001 Total pop
+#B03002_003 White Not Hispanic or Latino</t>
   </si>
 </sst>
 </file>
@@ -1217,10 +1214,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1983,7 +1976,7 @@
         <v>72</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>65</v>
@@ -1995,7 +1988,7 @@
         <v>66</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="170" x14ac:dyDescent="0.2">
@@ -2003,19 +1996,19 @@
         <v>73</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>65</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>43</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="187" x14ac:dyDescent="0.2">
@@ -2023,19 +2016,19 @@
         <v>74</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>65</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>43</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="102" x14ac:dyDescent="0.2">
@@ -2043,19 +2036,19 @@
         <v>30</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>65</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="306" x14ac:dyDescent="0.2">
@@ -2063,10 +2056,10 @@
         <v>78</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>67</v>
@@ -2075,10 +2068,10 @@
         <v>66</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="85" x14ac:dyDescent="0.2">
@@ -2086,10 +2079,10 @@
         <v>77</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>67</v>
@@ -2098,10 +2091,10 @@
         <v>66</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="119" x14ac:dyDescent="0.2">
@@ -2109,10 +2102,10 @@
         <v>75</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>67</v>
@@ -2121,10 +2114,10 @@
         <v>66</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="119" x14ac:dyDescent="0.2">
@@ -2132,10 +2125,10 @@
         <v>76</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>67</v>
@@ -2144,10 +2137,10 @@
         <v>66</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="102" x14ac:dyDescent="0.2">
@@ -2155,19 +2148,19 @@
         <v>79</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>51</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="187" x14ac:dyDescent="0.2">
@@ -2175,10 +2168,10 @@
         <v>80</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>67</v>
@@ -2187,10 +2180,10 @@
         <v>66</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="187" x14ac:dyDescent="0.2">
@@ -2198,10 +2191,10 @@
         <v>81</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>67</v>
@@ -2210,10 +2203,10 @@
         <v>66</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="102" x14ac:dyDescent="0.2">
@@ -2233,10 +2226,10 @@
         <v>66</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="102" x14ac:dyDescent="0.2">
@@ -2244,10 +2237,10 @@
         <v>83</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>67</v>
@@ -2256,10 +2249,10 @@
         <v>66</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="102" x14ac:dyDescent="0.2">
@@ -2267,10 +2260,10 @@
         <v>84</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>67</v>
@@ -2279,10 +2272,10 @@
         <v>66</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="85" x14ac:dyDescent="0.2">
@@ -2290,10 +2283,10 @@
         <v>85</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>117</v>
+        <v>161</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>67</v>
@@ -2302,10 +2295,10 @@
         <v>66</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>109</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="85" x14ac:dyDescent="0.2">
@@ -2313,10 +2306,10 @@
         <v>86</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>67</v>
@@ -2325,10 +2318,10 @@
         <v>66</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="85" x14ac:dyDescent="0.2">
@@ -2336,10 +2329,10 @@
         <v>87</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>67</v>
@@ -2348,10 +2341,10 @@
         <v>66</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="85" x14ac:dyDescent="0.2">
@@ -2359,10 +2352,10 @@
         <v>88</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D20" s="7" t="s">
         <v>67</v>
@@ -2371,10 +2364,10 @@
         <v>66</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="85" x14ac:dyDescent="0.2">
@@ -2382,10 +2375,10 @@
         <v>89</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>67</v>
@@ -2394,10 +2387,10 @@
         <v>66</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="85" x14ac:dyDescent="0.2">
@@ -2405,10 +2398,10 @@
         <v>90</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>67</v>
@@ -2417,10 +2410,10 @@
         <v>66</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="85" x14ac:dyDescent="0.2">
@@ -2428,10 +2421,10 @@
         <v>91</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D23" s="7" t="s">
         <v>67</v>
@@ -2440,10 +2433,10 @@
         <v>66</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="85" x14ac:dyDescent="0.2">
@@ -2451,10 +2444,10 @@
         <v>92</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D24" s="7" t="s">
         <v>67</v>
@@ -2463,10 +2456,10 @@
         <v>66</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="102" x14ac:dyDescent="0.2">
@@ -2474,19 +2467,19 @@
         <v>93</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>65</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>47</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="102" x14ac:dyDescent="0.2">
@@ -2494,30 +2487,30 @@
         <v>94</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>65</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>47</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="409.6" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>95</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D27" s="7" t="s">
         <v>67</v>
@@ -2526,10 +2519,10 @@
         <v>66</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="119" x14ac:dyDescent="0.2">
@@ -2537,27 +2530,27 @@
         <v>96</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E28" s="2">
         <v>2019</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="119" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>97</v>
+        <v>7</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>7</v>
@@ -2566,16 +2559,16 @@
         <v>65</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E29" s="2">
         <v>2018</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="85" x14ac:dyDescent="0.2">
@@ -2583,10 +2576,10 @@
         <v>57</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>67</v>
@@ -2595,10 +2588,10 @@
         <v>66</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
udpate HVI var_def as per v1.1 dashbaord release #32
</commit_message>
<xml_diff>
--- a/Data/data documentation/Data documentation for council variables.xlsx
+++ b/Data/data documentation/Data documentation for council variables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://drexel0-my.sharepoint.com/personal/tr842_drexel_edu/Documents/Github_repositories/philadelphia-council-districts-and-health/Data/data documentation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranli\Documents\GitHub\philadelphia-council-districts-and-health\Data\data documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{01B3F741-F830-43A2-8E49-C5302E8723C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D2CF2A3-1FAC-AB46-9E38-E583BFA9D6A2}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C06779E5-6FD9-4282-83E7-1A1FDC362FD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6600" yWindow="2760" windowWidth="23260" windowHeight="12460" activeTab="1" xr2:uid="{7E76C4D9-7630-4340-BEBA-4E6127603C3B}"/>
+    <workbookView xWindow="54960" yWindow="1365" windowWidth="18900" windowHeight="10890" activeTab="1" xr2:uid="{7E76C4D9-7630-4340-BEBA-4E6127603C3B}"/>
   </bookViews>
   <sheets>
     <sheet name="Data documentation for council " sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="164">
   <si>
     <t>Map</t>
   </si>
@@ -622,6 +622,9 @@
     <t>Variables Used:
 #B02001_001 Total pop
 #B03002_003 White Not Hispanic or Latino</t>
+  </si>
+  <si>
+    <t>The Heat Vulnerability Index (HVI) is a composite measure that summarizes key indicators associated with negative health outcomes due to extreme heat exposure. The HVI scale ranges from negative to positive values, which represent areas of very low to very high vulnerability.</t>
   </si>
 </sst>
 </file>
@@ -1534,18 +1537,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01CB8890-B7A9-3A40-979C-A48DC9A37105}">
   <dimension ref="A1:H27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.33203125" customWidth="1"/>
-    <col min="6" max="6" width="27.1640625" customWidth="1"/>
-    <col min="7" max="7" width="15.1640625" customWidth="1"/>
+    <col min="2" max="2" width="20.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.296875" customWidth="1"/>
+    <col min="6" max="6" width="27.19921875" customWidth="1"/>
+    <col min="7" max="7" width="15.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1568,7 +1571,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1591,7 +1594,7 @@
         <v>45716</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="289" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" ht="265.2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1614,7 +1617,7 @@
         <v>45725</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="388" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" ht="358.8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -1637,7 +1640,7 @@
         <v>45726</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="204" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -1660,7 +1663,7 @@
         <v>45718</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -1683,7 +1686,7 @@
         <v>45719</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>27</v>
       </c>
@@ -1706,7 +1709,7 @@
         <v>45719</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -1729,7 +1732,7 @@
         <v>45719</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>35</v>
       </c>
@@ -1749,7 +1752,7 @@
         <v>45719</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>38</v>
       </c>
@@ -1772,7 +1775,7 @@
         <v>45725</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -1795,7 +1798,7 @@
         <v>45725</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>46</v>
       </c>
@@ -1818,7 +1821,7 @@
         <v>45726</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>50</v>
       </c>
@@ -1841,7 +1844,7 @@
         <v>45725</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="323" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" ht="296.39999999999998" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>54</v>
       </c>
@@ -1864,7 +1867,7 @@
         <v>45726</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="221" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>57</v>
       </c>
@@ -1887,7 +1890,7 @@
         <v>45726</v>
       </c>
     </row>
-    <row r="26" spans="1:8" s="5" customFormat="1" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" s="5" customFormat="1" ht="19.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -1897,7 +1900,7 @@
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -1915,17 +1918,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B07AACCA-88DB-7C45-AECA-8998520502A5}">
   <dimension ref="A1:G30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.1640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="20.33203125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="22.33203125" style="2" customWidth="1"/>
-    <col min="4" max="5" width="11.1640625" style="2"/>
-    <col min="6" max="6" width="19.6640625" customWidth="1"/>
+    <col min="1" max="1" width="20.19921875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="20.296875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.296875" style="2" customWidth="1"/>
+    <col min="4" max="5" width="11.19921875" style="2"/>
+    <col min="6" max="6" width="19.69921875" customWidth="1"/>
     <col min="7" max="7" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>60</v>
       </c>
@@ -1948,7 +1951,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>20</v>
       </c>
@@ -1971,7 +1974,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>72</v>
       </c>
@@ -1991,7 +1994,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="170" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" ht="156" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>73</v>
       </c>
@@ -2011,7 +2014,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="187" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>74</v>
       </c>
@@ -2031,7 +2034,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="102" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>30</v>
       </c>
@@ -2051,7 +2054,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="306" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" ht="280.8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>78</v>
       </c>
@@ -2074,7 +2077,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>77</v>
       </c>
@@ -2097,7 +2100,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="119" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" ht="109.2" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>75</v>
       </c>
@@ -2120,7 +2123,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="119" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" ht="109.2" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>76</v>
       </c>
@@ -2143,7 +2146,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="102" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>79</v>
       </c>
@@ -2163,7 +2166,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="187" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>80</v>
       </c>
@@ -2186,7 +2189,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="187" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>81</v>
       </c>
@@ -2209,7 +2212,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="102" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>82</v>
       </c>
@@ -2232,7 +2235,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="102" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>83</v>
       </c>
@@ -2255,7 +2258,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="102" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>84</v>
       </c>
@@ -2278,7 +2281,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>85</v>
       </c>
@@ -2301,7 +2304,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>86</v>
       </c>
@@ -2324,7 +2327,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>87</v>
       </c>
@@ -2347,7 +2350,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>88</v>
       </c>
@@ -2370,7 +2373,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>89</v>
       </c>
@@ -2393,7 +2396,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>90</v>
       </c>
@@ -2416,7 +2419,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>91</v>
       </c>
@@ -2439,7 +2442,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>92</v>
       </c>
@@ -2462,7 +2465,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="102" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>93</v>
       </c>
@@ -2482,7 +2485,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="102" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>94</v>
       </c>
@@ -2502,7 +2505,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="409.5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>95</v>
       </c>
@@ -2525,7 +2528,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="119" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" ht="109.2" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>96</v>
       </c>
@@ -2548,12 +2551,12 @@
         <v>142</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="119" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" ht="109.2" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>7</v>
+      <c r="B29" t="s">
+        <v>163</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>65</v>
@@ -2571,7 +2574,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>57</v>
       </c>

</xml_diff>